<commit_message>
Fix lỗi xuất ra file excel thay vì csv trong tồn đầu kỳ, thêm nút xóa đồng loạt các mục được chọn trong phần danh mục và khai báo tồn kho đầu kỳ.
</commit_message>
<xml_diff>
--- a/docs/Ton dau ky/file ton kho dau ky mau..xlsx
+++ b/docs/Ton dau ky/file ton kho dau ky mau..xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!Project\Zencos_NVL\docs\Ton dau ky\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{44629ECE-E961-46D9-8830-A7CAD3C9D595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37261F2E-7703-4657-B792-1CECBBB33F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="107">
   <si>
     <t>STT</t>
   </si>
@@ -324,48 +324,6 @@
     <t>NL-PGI-040</t>
   </si>
   <si>
-    <t>HD_MIFA_1361</t>
-  </si>
-  <si>
-    <t>HD_HOAN VU_11</t>
-  </si>
-  <si>
-    <t>HD_KHANGNGOC_638</t>
-  </si>
-  <si>
-    <t>HD_KHANGNGOC_997</t>
-  </si>
-  <si>
-    <t>HD_3H_723</t>
-  </si>
-  <si>
-    <t>HD_NGUYENBA_9911</t>
-  </si>
-  <si>
-    <t>HD_NGUYENBA_12118</t>
-  </si>
-  <si>
-    <t>HD_DERMATRIX_35</t>
-  </si>
-  <si>
-    <t>HD_HOANVU_24</t>
-  </si>
-  <si>
-    <t>HD_CHEMICO_2911</t>
-  </si>
-  <si>
-    <t>HD_CHEMICO_3120</t>
-  </si>
-  <si>
-    <t>HD_CHEMICO_2557</t>
-  </si>
-  <si>
-    <t>HD_NGUYENBA_1829</t>
-  </si>
-  <si>
-    <t>HD_SMALLFORTUNE_8164</t>
-  </si>
-  <si>
     <t>HƯƠNG</t>
   </si>
   <si>
@@ -390,104 +348,7 @@
     <t>ĐƠN GIÁ</t>
   </si>
   <si>
-    <t>MSDS_COA_PROPYLENE GLYCOL</t>
-  </si>
-  <si>
-    <t>COA_PROPYLENE GLYCOL_GX250204L1</t>
-  </si>
-  <si>
-    <t>MSDS_GLYCERIN</t>
-  </si>
-  <si>
-    <t>COA_GLYCERIN_014125IND3C5L</t>
-  </si>
-  <si>
     <t>KHÁC</t>
-  </si>
-  <si>
-    <t>TEST REPORT_GLYCERIN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COA_ALLANTOIN_25LOT01156
-</t>
-  </si>
-  <si>
-    <t>MSDS_ALLANTOIN</t>
-  </si>
-  <si>
-    <t>COA_D-PANTHENOL_TL02409085,COA_D-PANTHENOL_TL02409085</t>
-  </si>
-  <si>
-    <t>COA_CS-GINGER EXT_EI2501</t>
-  </si>
-  <si>
-    <t>MSDS_CS-GINGER EXT</t>
-  </si>
-  <si>
-    <t>COA_RICOBIO JA7_25091685</t>
-  </si>
-  <si>
-    <t>MSDS_RICOBIO JA7</t>
-  </si>
-  <si>
-    <t>MSDS_CARBOMER</t>
-  </si>
-  <si>
-    <t>COA_CARBOMER_B2E04349</t>
-  </si>
-  <si>
-    <t>COA_CARBOMER_B2F04120</t>
-  </si>
-  <si>
-    <t>COA_VITAMIN E_32666436W0</t>
-  </si>
-  <si>
-    <t>MSDS_VITAMINE</t>
-  </si>
-  <si>
-    <t>COA_TOCOPHERYL ACETATE_UT25100294</t>
-  </si>
-  <si>
-    <t>MSDS_TOCOPHERYL ACETATE</t>
-  </si>
-  <si>
-    <t>COA_METHYL SALICYLATE_2502009</t>
-  </si>
-  <si>
-    <t>MSDS_METHYL SALICYLATE</t>
-  </si>
-  <si>
-    <t>MSDS_HOT FLUX</t>
-  </si>
-  <si>
-    <t>COA_HOT FLUX_AT117926</t>
-  </si>
-  <si>
-    <t>COA_HOT FLUX_AT115815</t>
-  </si>
-  <si>
-    <t>COA_EHGP_AT115815</t>
-  </si>
-  <si>
-    <t>MSDS_EHGP_THOR</t>
-  </si>
-  <si>
-    <t>COA_EHGP_IP13130</t>
-  </si>
-  <si>
-    <t>MSDS_EHGP_ISCA</t>
-  </si>
-  <si>
-    <t>COA_COSMAN CR530_20250228</t>
-  </si>
-  <si>
-    <t>MSDS_COSMAN CR530</t>
-  </si>
-  <si>
-    <t>COA_TRIETHANOLAMINE_71353A</t>
-  </si>
-  <si>
-    <t>MSDS_TRIETHANOLAMINE</t>
   </si>
 </sst>
 </file>
@@ -1007,7 +868,7 @@
         <v>58</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>68</v>
@@ -1016,10 +877,10 @@
         <v>69</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="K1" s="6" t="s">
         <v>70</v>
@@ -1037,16 +898,16 @@
         <v>29</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="R1" s="6" t="s">
         <v>71</v>
       </c>
       <c r="S1" s="6" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:19" s="8" customFormat="1" ht="96.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -1066,7 +927,7 @@
         <v>202000</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G2" s="29">
         <v>1361</v>
@@ -1078,7 +939,7 @@
         <v>34100</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K2" s="20">
         <f>E2/1000*I2</f>
@@ -1096,15 +957,9 @@
       <c r="O2" s="24">
         <v>46350</v>
       </c>
-      <c r="P2" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q2" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="R2" s="41" t="s">
-        <v>98</v>
-      </c>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="41"/>
       <c r="S2" s="11"/>
     </row>
     <row r="3" spans="1:19" s="8" customFormat="1" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1124,7 +979,7 @@
         <v>50401.279999999999</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G3" s="29">
         <v>11</v>
@@ -1136,7 +991,7 @@
         <v>33000</v>
       </c>
       <c r="J3" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K3" s="20">
         <f>E3/1000*I3</f>
@@ -1154,15 +1009,9 @@
       <c r="O3" s="24">
         <v>46472</v>
       </c>
-      <c r="P3" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q3" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="R3" s="41" t="s">
-        <v>99</v>
-      </c>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="41"/>
       <c r="S3" s="11"/>
     </row>
     <row r="4" spans="1:19" s="8" customFormat="1" ht="93" customHeight="1" x14ac:dyDescent="0.25">
@@ -1182,7 +1031,7 @@
         <v>117000</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G4" s="29">
         <v>1361</v>
@@ -1194,7 +1043,7 @@
         <v>34000</v>
       </c>
       <c r="J4" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K4" s="20">
         <f>E4/1000*I4</f>
@@ -1212,16 +1061,10 @@
       <c r="O4" s="24">
         <v>46378</v>
       </c>
-      <c r="P4" s="10" t="s">
-        <v>122</v>
-      </c>
+      <c r="P4" s="10"/>
       <c r="Q4" s="11"/>
-      <c r="R4" s="41" t="s">
-        <v>98</v>
-      </c>
-      <c r="S4" s="11" t="s">
-        <v>125</v>
-      </c>
+      <c r="R4" s="41"/>
+      <c r="S4" s="11"/>
     </row>
     <row r="5" spans="1:19" s="8" customFormat="1" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
@@ -1240,13 +1083,13 @@
         <v>0</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G5" s="29"/>
       <c r="H5" s="34"/>
       <c r="I5" s="20"/>
       <c r="J5" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K5" s="20"/>
       <c r="L5" s="10"/>
@@ -1255,9 +1098,7 @@
       <c r="O5" s="24"/>
       <c r="P5" s="10"/>
       <c r="Q5" s="11"/>
-      <c r="R5" s="42" t="s">
-        <v>100</v>
-      </c>
+      <c r="R5" s="42"/>
       <c r="S5" s="11"/>
     </row>
     <row r="6" spans="1:19" s="8" customFormat="1" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1277,7 +1118,7 @@
         <v>5186.8</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G6" s="29">
         <v>11</v>
@@ -1289,7 +1130,7 @@
         <v>260000</v>
       </c>
       <c r="J6" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K6" s="20">
         <f t="shared" ref="K6:K19" si="0">E6/1000*I6</f>
@@ -1307,15 +1148,9 @@
       <c r="O6" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="P6" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="Q6" s="17" t="s">
-        <v>126</v>
-      </c>
-      <c r="R6" s="41" t="s">
-        <v>99</v>
-      </c>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="41"/>
       <c r="S6" s="11"/>
     </row>
     <row r="7" spans="1:19" s="8" customFormat="1" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1335,7 +1170,7 @@
         <v>35572</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G7" s="29">
         <v>1361</v>
@@ -1347,7 +1182,7 @@
         <v>430556</v>
       </c>
       <c r="J7" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K7" s="20">
         <f t="shared" si="0"/>
@@ -1366,12 +1201,8 @@
         <v>46649</v>
       </c>
       <c r="P7" s="10"/>
-      <c r="Q7" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="R7" s="42" t="s">
-        <v>98</v>
-      </c>
+      <c r="Q7" s="11"/>
+      <c r="R7" s="42"/>
       <c r="S7" s="11"/>
     </row>
     <row r="8" spans="1:19" s="8" customFormat="1" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1391,7 +1222,7 @@
         <v>200</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G8" s="29">
         <v>997</v>
@@ -1403,7 +1234,7 @@
         <v>2450000</v>
       </c>
       <c r="J8" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K8" s="20">
         <f t="shared" si="0"/>
@@ -1421,15 +1252,9 @@
       <c r="O8" s="24">
         <v>46654</v>
       </c>
-      <c r="P8" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="Q8" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="R8" s="42" t="s">
-        <v>101</v>
-      </c>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="11"/>
+      <c r="R8" s="42"/>
       <c r="S8" s="11"/>
     </row>
     <row r="9" spans="1:19" s="8" customFormat="1" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1449,7 +1274,7 @@
         <v>192</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G9" s="29">
         <v>723</v>
@@ -1461,7 +1286,7 @@
         <v>3000000</v>
       </c>
       <c r="J9" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K9" s="20">
         <f t="shared" si="0"/>
@@ -1479,15 +1304,9 @@
       <c r="O9" s="24">
         <v>46645</v>
       </c>
-      <c r="P9" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="Q9" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="R9" s="42" t="s">
-        <v>102</v>
-      </c>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="42"/>
       <c r="S9" s="11"/>
     </row>
     <row r="10" spans="1:19" s="8" customFormat="1" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
@@ -1507,7 +1326,7 @@
         <v>2000</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G10" s="30">
         <v>9911</v>
@@ -1519,7 +1338,7 @@
         <v>351852</v>
       </c>
       <c r="J10" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K10" s="20">
         <f t="shared" si="0"/>
@@ -1537,15 +1356,9 @@
       <c r="O10" s="24">
         <v>46418</v>
       </c>
-      <c r="P10" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="Q10" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="R10" s="42" t="s">
-        <v>103</v>
-      </c>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="42"/>
       <c r="S10" s="11"/>
     </row>
     <row r="11" spans="1:19" s="8" customFormat="1" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1565,7 +1378,7 @@
         <v>8300</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G11" s="30">
         <v>12118</v>
@@ -1577,7 +1390,7 @@
         <v>333333.34000000003</v>
       </c>
       <c r="J11" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K11" s="20">
         <f t="shared" si="0"/>
@@ -1595,15 +1408,9 @@
       <c r="O11" s="24">
         <v>46538</v>
       </c>
-      <c r="P11" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="Q11" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="R11" s="42" t="s">
-        <v>104</v>
-      </c>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="42"/>
       <c r="S11" s="11"/>
     </row>
     <row r="12" spans="1:19" s="8" customFormat="1" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1620,7 +1427,7 @@
         <v>8</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G12" s="30">
         <v>35</v>
@@ -1632,7 +1439,7 @@
         <v>302400</v>
       </c>
       <c r="J12" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K12" s="20">
         <f>E11/1000*I12</f>
@@ -1646,9 +1453,7 @@
       <c r="O12" s="24"/>
       <c r="P12" s="10"/>
       <c r="Q12" s="11"/>
-      <c r="R12" s="42" t="s">
-        <v>105</v>
-      </c>
+      <c r="R12" s="42"/>
       <c r="S12" s="11"/>
     </row>
     <row r="13" spans="1:19" s="8" customFormat="1" ht="76.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1668,7 +1473,7 @@
         <v>32674.799999999999</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G13" s="29">
         <v>1361</v>
@@ -1680,7 +1485,7 @@
         <v>584259</v>
       </c>
       <c r="J13" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K13" s="20">
         <f t="shared" si="0"/>
@@ -1698,15 +1503,9 @@
       <c r="O13" s="24">
         <v>46423</v>
       </c>
-      <c r="P13" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="Q13" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="R13" s="42" t="s">
-        <v>98</v>
-      </c>
+      <c r="P13" s="10"/>
+      <c r="Q13" s="11"/>
+      <c r="R13" s="42"/>
       <c r="S13" s="11"/>
     </row>
     <row r="14" spans="1:19" s="8" customFormat="1" ht="81" customHeight="1" x14ac:dyDescent="0.25">
@@ -1726,7 +1525,7 @@
         <v>20000</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G14" s="29">
         <v>24</v>
@@ -1738,7 +1537,7 @@
         <v>800000</v>
       </c>
       <c r="J14" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K14" s="20">
         <f t="shared" si="0"/>
@@ -1756,15 +1555,9 @@
       <c r="O14" s="24">
         <v>47388</v>
       </c>
-      <c r="P14" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q14" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="R14" s="42" t="s">
-        <v>106</v>
-      </c>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="11"/>
+      <c r="R14" s="42"/>
       <c r="S14" s="11"/>
     </row>
     <row r="15" spans="1:19" s="8" customFormat="1" ht="89.55" customHeight="1" x14ac:dyDescent="0.25">
@@ -1784,7 +1577,7 @@
         <v>4000</v>
       </c>
       <c r="F15" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G15" s="29">
         <v>12118</v>
@@ -1796,7 +1589,7 @@
         <v>180555.56</v>
       </c>
       <c r="J15" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K15" s="20">
         <f t="shared" si="0"/>
@@ -1814,15 +1607,9 @@
       <c r="O15" s="24">
         <v>46789</v>
       </c>
-      <c r="P15" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="Q15" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="R15" s="42" t="s">
-        <v>104</v>
-      </c>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="11"/>
+      <c r="R15" s="42"/>
       <c r="S15" s="11"/>
     </row>
     <row r="16" spans="1:19" s="8" customFormat="1" ht="79.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1842,7 +1629,7 @@
         <v>6000</v>
       </c>
       <c r="F16" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G16" s="29">
         <v>2911</v>
@@ -1854,7 +1641,7 @@
         <v>10296390</v>
       </c>
       <c r="J16" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K16" s="20">
         <f t="shared" si="0"/>
@@ -1872,15 +1659,9 @@
       <c r="O16" s="24">
         <v>46514</v>
       </c>
-      <c r="P16" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="Q16" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="R16" s="42" t="s">
-        <v>107</v>
-      </c>
+      <c r="P16" s="10"/>
+      <c r="Q16" s="11"/>
+      <c r="R16" s="42"/>
       <c r="S16" s="11"/>
     </row>
     <row r="17" spans="1:19" s="8" customFormat="1" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1900,7 +1681,7 @@
         <v>2000</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G17" s="29">
         <v>3120</v>
@@ -1912,7 +1693,7 @@
         <v>10427210</v>
       </c>
       <c r="J17" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K17" s="20">
         <f t="shared" si="0"/>
@@ -1930,15 +1711,9 @@
       <c r="O17" s="24">
         <v>46591</v>
       </c>
-      <c r="P17" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="Q17" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="R17" s="42" t="s">
-        <v>108</v>
-      </c>
+      <c r="P17" s="10"/>
+      <c r="Q17" s="11"/>
+      <c r="R17" s="42"/>
       <c r="S17" s="11"/>
     </row>
     <row r="18" spans="1:19" s="8" customFormat="1" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1958,7 +1733,7 @@
         <v>31368.9</v>
       </c>
       <c r="F18" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G18" s="29">
         <v>2557</v>
@@ -1970,7 +1745,7 @@
         <v>250505.5</v>
       </c>
       <c r="J18" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K18" s="20">
         <f t="shared" si="0"/>
@@ -1988,15 +1763,9 @@
       <c r="O18" s="25">
         <v>46459</v>
       </c>
-      <c r="P18" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="Q18" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="R18" s="42" t="s">
-        <v>109</v>
-      </c>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="11"/>
+      <c r="R18" s="42"/>
       <c r="S18" s="11"/>
     </row>
     <row r="19" spans="1:19" s="8" customFormat="1" ht="76.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2016,7 +1785,7 @@
         <v>12000</v>
       </c>
       <c r="F19" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G19" s="29">
         <v>1361</v>
@@ -2028,7 +1797,7 @@
         <v>257000</v>
       </c>
       <c r="J19" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K19" s="20">
         <f t="shared" si="0"/>
@@ -2046,15 +1815,9 @@
       <c r="O19" s="25">
         <v>46223</v>
       </c>
-      <c r="P19" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q19" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="R19" s="42" t="s">
-        <v>98</v>
-      </c>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="11"/>
+      <c r="R19" s="42"/>
       <c r="S19" s="11"/>
     </row>
     <row r="20" spans="1:19" s="8" customFormat="1" ht="52.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2068,17 +1831,17 @@
         <v>19</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="E20" s="20"/>
       <c r="F20" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G20" s="29"/>
       <c r="H20" s="34"/>
       <c r="I20" s="20"/>
       <c r="J20" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K20" s="20"/>
       <c r="L20" s="10"/>
@@ -2107,7 +1870,7 @@
         <v>1000</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G21" s="29">
         <v>1829</v>
@@ -2119,7 +1882,7 @@
         <v>800000</v>
       </c>
       <c r="J21" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K21" s="20">
         <f>E21/1000*I21</f>
@@ -2137,15 +1900,9 @@
       <c r="O21" s="27">
         <v>46445</v>
       </c>
-      <c r="P21" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="Q21" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="R21" s="42" t="s">
-        <v>110</v>
-      </c>
+      <c r="P21" s="10"/>
+      <c r="Q21" s="11"/>
+      <c r="R21" s="42"/>
       <c r="S21" s="11"/>
     </row>
     <row r="22" spans="1:19" s="8" customFormat="1" ht="78.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2165,7 +1922,7 @@
         <v>13991</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G22" s="29">
         <v>8164</v>
@@ -2177,7 +1934,7 @@
         <v>50926</v>
       </c>
       <c r="J22" s="20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K22" s="20">
         <f>E22/1000*I22</f>
@@ -2195,15 +1952,9 @@
       <c r="O22" s="24">
         <v>46558</v>
       </c>
-      <c r="P22" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="Q22" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="R22" s="42" t="s">
-        <v>111</v>
-      </c>
+      <c r="P22" s="10"/>
+      <c r="Q22" s="11"/>
+      <c r="R22" s="42"/>
       <c r="S22" s="11"/>
     </row>
     <row r="23" spans="1:19" s="8" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">

</xml_diff>